<commit_message>
Selfi printer v4: dæmpeplade med knusekegler, gribehak i begge ender og slanke vægkonsoller
Printeren står på en printet dæmpeplade med 56 hule kegler i 2 ringe ved
kanten (2 mm-bunden bøjer ellers), kegler på kappens endevæg og udgangs-
modulets bøjler. Lukkede gribehak (76 × 22, loftet 20° op indad) i kappens
venstre ende og udgangsmodulets højre ende. Vægkonsollerne er T-arme med
110 mm bagplade (63 % mindre plast). Soklens skruer 4,0 × 16, tungens
skruer nedefra. Nye printfiler, 3D, tegning, indkøbsliste, printguide og
hurtigsæt; hjemmesidens printer er nu v4.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQrVqPvEFmrvZ9rajYjAFd
</commit_message>
<xml_diff>
--- a/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
+++ b/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -915,7 +915,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Skrue til plast 3,5 × 10, undersænket (fx Spax)</t>
+          <t>Skrue til plast 3,5 × 12, undersænket (fx Spax)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sokkel → udgangsmodulets tunge</t>
+          <t>Soklens tunge → udgangsmodulet, nedefra</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -946,7 +946,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPUN+ Climate 4,0 × 30, undersænket</t>
+          <t>SPUN+ Climate 4,0 × 16, undersænket</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Sokkel → bord eller hylde (under printeren)</t>
+          <t>Sokkel → bord, hylde eller konsol: sættes i før dæmpepladen</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1165,7 +1165,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Kappe med låsehul (flad top, lameller, 6 kroge)</t>
+          <t>Kappe med låsehul (flad top, lameller, 6 kroge, knusekegler ved enden)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1174,13 +1174,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>750</v>
+        <v>760</v>
       </c>
       <c r="D27" t="n">
         <v>0.25</v>
       </c>
       <c r="E27" t="n">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sokkel under printeren (kabelspor, rille til skumsnor, krog-ramper)</t>
+          <t>Sokkel under printeren (kabelspor, rille til skumsnor, krog-ramper, lomme til dæmpepladen)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1252,13 +1252,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>475</v>
+        <v>300</v>
       </c>
       <c r="D30" t="n">
         <v>0.25</v>
       </c>
       <c r="E30" t="n">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Udgangsmodul (papirrum, rutsjebane, lomme, skærm, LED-skinne)</t>
+          <t>Dæmpeplade med 56 knusekegler (udskiftes efter et hårdt fald)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1278,13 +1278,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>905</v>
+        <v>85</v>
       </c>
       <c r="D31" t="n">
         <v>0.25</v>
       </c>
       <c r="E31" t="n">
-        <v>226</v>
+        <v>21</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1295,22 +1295,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2 vægkonsoller</t>
+          <t>Udgangsmodul (papirrum, rutsjebane, lomme, skærm, LED-skinne, knusekegler)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>B2B væg</t>
+          <t>Alle</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1300</v>
+        <v>960</v>
       </c>
       <c r="D32" t="n">
         <v>0.25</v>
       </c>
       <c r="E32" t="n">
-        <v>325</v>
+        <v>240</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2 vægskinner</t>
+          <t>2 vægkonsoller, slanke T-arme</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1330,13 +1330,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>300</v>
+        <v>520</v>
       </c>
       <c r="D33" t="n">
         <v>0.25</v>
       </c>
       <c r="E33" t="n">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1344,67 +1344,93 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2 vægskinner</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>B2B væg</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>150</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E34" t="n">
+        <v>38</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>sort ASA</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Sum</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Printer-pakke B2C (bord)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>9875</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>inkl. begge ruller</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>B2B (bord/disk, skruet fast)</t>
+          <t>Printer-pakke B2C (bord)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>9879</v>
+        <v>9868</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>+ 2 skruer</t>
+          <t>inkl. begge ruller</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>B2B væg</t>
+          <t>B2B (bord/disk, skruet fast)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>10323</v>
+        <v>9872</v>
       </c>
       <c r="F38" t="inlineStr">
+        <is>
+          <t>+ 2 skruer</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>B2B væg</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>10084</v>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>+ 2 konsoller, 2 vægskinner og skruer</t>
         </is>

</xml_diff>

<commit_message>
Printer v4: brede, symmetriske vægkonsoller (hylde 200, 20 mm inde fra hver ende, 110 høj)
Hylderne har samme bredde som i v3 igen og står symmetrisk under printeren.
Knægte 6 mm i hver side, 2 vinduer i hylden, vægskinne 160 bred.
Vægskruernes retning i 3D rettet (de gik ind i konsollen).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQrVqPvEFmrvZ9rajYjAFd
</commit_message>
<xml_diff>
--- a/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
+++ b/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
@@ -1321,7 +1321,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2 vægkonsoller, slanke T-arme</t>
+          <t>2 vægkonsoller, hylder 200 brede</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1330,13 +1330,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>520</v>
+        <v>680</v>
       </c>
       <c r="D33" t="n">
         <v>0.25</v>
       </c>
       <c r="E33" t="n">
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1428,7 +1428,7 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>10084</v>
+        <v>10124</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Printer v4: skjulte L-beslag i stedet for konsoller med knægte
Esben: knægtene er for synlige. 2 ens L-beslag (238 lange, samlet med 2
dyvelstifter): hylde 15 under printeren, bagplade 15 bag den, skruet i
væggen dér, så kun hyldens kant ses. Ingen vægskinner eller
sikkerhedsskruer. Printes på enden; ca. 7 MPa i hjørnet ved 500 N.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQrVqPvEFmrvZ9rajYjAFd
</commit_message>
<xml_diff>
--- a/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
+++ b/hardware/stl/printer/selfi-printer-v4/selfi-printer-v4_indkoebsliste.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1039,7 +1039,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SPUN+ Climate 4,0 × 20, undersænket</t>
+          <t>SPUN+ Climate 4,0 × 25, undersænket</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Højre konsol → udgangsmodulet (nedefra)</t>
+          <t>Højre L-beslag → udgangsmodulet (nedefra)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2 vægskinner, 4 hver</t>
+          <t>2 L-beslag, 4 hver, skjult bag printeren. I gips: metal-gipsdybler eller skru i en lægte</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sikkerhedsskrue Torx med pind 4,0 × 25 + bit</t>
+          <t>Dyvelstift Ø6 × 16, stål</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1113,14 +1113,14 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Konsol → vægskinne, så konsollen ikke kan løftes af</t>
+          <t>Samler de 2 L-beslag i enderne, så de sidder i lige linje og samme højde</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2 vægkonsoller, hylder 200 brede</t>
+          <t>2 skjulte L-beslag (hylde under printeren, bagplade bag den)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1330,13 +1330,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>680</v>
+        <v>900</v>
       </c>
       <c r="D33" t="n">
         <v>0.25</v>
       </c>
       <c r="E33" t="n">
-        <v>170</v>
+        <v>225</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1344,95 +1344,69 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2 vægskinner</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>150</v>
-      </c>
-      <c r="D34" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E34" t="n">
-        <v>38</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>sort ASA</t>
-        </is>
-      </c>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Sum</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Printer-pakke B2C (bord)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>9868</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>inkl. begge ruller</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Printer-pakke B2C (bord)</t>
+          <t>B2B (bord/disk, skruet fast)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
-        <v>9868</v>
+        <v>9872</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inkl. begge ruller</t>
+          <t>+ 2 skruer</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>B2B (bord/disk, skruet fast)</t>
+          <t>B2B væg</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>9872</v>
+        <v>10130</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>+ 2 skruer</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>B2B væg</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="n">
-        <v>10124</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>+ 2 konsoller, 2 vægskinner og skruer</t>
+          <t>+ 2 L-beslag og skruer</t>
         </is>
       </c>
     </row>

</xml_diff>